<commit_message>
feat: implementacion de carga masiva de proyectos desde excel
</commit_message>
<xml_diff>
--- a/ejecucion.xlsx
+++ b/ejecucion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prueb\OneDrive\Documentos\GIRA\2026\PARTICIPACION\pp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7AB183-C11B-412B-B028-EA0BAB0B81F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34ABE792-CACA-40A5-93C8-05F391E148AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6C8ED67E-9047-42B1-8BDB-DD58B52646C4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{6C8ED67E-9047-42B1-8BDB-DD58B52646C4}"/>
   </bookViews>
   <sheets>
     <sheet name="2024" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="233">
   <si>
     <t>Barrio o vereda</t>
   </si>
@@ -620,51 +620,6 @@
     <t>LICITACIÓN</t>
   </si>
   <si>
-    <t>MATICA PARTE BAJA</t>
-  </si>
-  <si>
-    <t>ESTUDIO HIDROLOGICO</t>
-  </si>
-  <si>
-    <t>$100,000,000.00</t>
-  </si>
-  <si>
-    <t>Diseños,</t>
-  </si>
-  <si>
-    <t>CENTROS DE DESARROLLO COMUNITARIO</t>
-  </si>
-  <si>
-    <t>4 AÑOS</t>
-  </si>
-  <si>
-    <t>PORTACHUELO</t>
-  </si>
-  <si>
-    <t>2026-2027</t>
-  </si>
-  <si>
-    <t>JUAN C0JO</t>
-  </si>
-  <si>
-    <t>$310,000,000.00</t>
-  </si>
-  <si>
-    <t>CANO</t>
-  </si>
-  <si>
-    <t>Cubierta Placa Polideportiva</t>
-  </si>
-  <si>
-    <t>Ampliación Sede</t>
-  </si>
-  <si>
-    <t>COMPRA</t>
-  </si>
-  <si>
-    <t>SAN JOSE</t>
-  </si>
-  <si>
     <t>Cerramiento</t>
   </si>
   <si>
@@ -794,9 +749,6 @@
     <t>2025-20206</t>
   </si>
   <si>
-    <t>Suministro</t>
-  </si>
-  <si>
     <t>Ajuste del 2024</t>
   </si>
   <si>
@@ -806,7 +758,7 @@
     <t>EXCEDENTE</t>
   </si>
   <si>
-    <t>MERCEDES ABREGO</t>
+    <t>PLANEACIÓN</t>
   </si>
 </sst>
 </file>
@@ -1374,7 +1326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1619,9 +1571,6 @@
     <xf numFmtId="165" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1801,33 +1750,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2508,7 +2430,7 @@
       <c r="O7" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="P7" s="121">
+      <c r="P7" s="120">
         <v>35697000</v>
       </c>
     </row>
@@ -2527,8 +2449,8 @@
       <c r="L8" s="19"/>
       <c r="M8" s="19"/>
       <c r="N8" s="19"/>
-      <c r="O8" s="120"/>
-      <c r="P8" s="123">
+      <c r="O8" s="119"/>
+      <c r="P8" s="122">
         <f>SUM(P2:P7)</f>
         <v>201218952</v>
       </c>
@@ -2549,7 +2471,7 @@
       <c r="M9" s="19"/>
       <c r="N9" s="19"/>
       <c r="O9" s="19"/>
-      <c r="P9" s="122"/>
+      <c r="P9" s="121"/>
     </row>
     <row r="10" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="20"/>
@@ -2570,15 +2492,15 @@
       <c r="P10" s="19"/>
     </row>
     <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="134" t="s">
+      <c r="A11" s="133" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="135"/>
-      <c r="C11" s="135"/>
-      <c r="D11" s="135"/>
-      <c r="E11" s="135"/>
-      <c r="F11" s="135"/>
-      <c r="G11" s="136"/>
+      <c r="B11" s="134"/>
+      <c r="C11" s="134"/>
+      <c r="D11" s="134"/>
+      <c r="E11" s="134"/>
+      <c r="F11" s="134"/>
+      <c r="G11" s="135"/>
       <c r="H11" s="19"/>
       <c r="I11" s="19"/>
       <c r="J11" s="19"/>
@@ -2814,34 +2736,34 @@
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="25.54296875" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" style="126"/>
+    <col min="6" max="6" width="11.453125" style="125"/>
     <col min="10" max="10" width="16" customWidth="1"/>
     <col min="20" max="20" width="17.54296875" customWidth="1"/>
     <col min="21" max="21" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="137"/>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="138"/>
-      <c r="O1" s="138"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="138"/>
-      <c r="R1" s="138"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="138"/>
-      <c r="U1" s="139"/>
+      <c r="A1" s="136"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
+      <c r="F1" s="137"/>
+      <c r="G1" s="137"/>
+      <c r="H1" s="137"/>
+      <c r="I1" s="137"/>
+      <c r="J1" s="137"/>
+      <c r="K1" s="137"/>
+      <c r="L1" s="137"/>
+      <c r="M1" s="137"/>
+      <c r="N1" s="137"/>
+      <c r="O1" s="137"/>
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="137"/>
+      <c r="U1" s="138"/>
       <c r="V1" s="26"/>
       <c r="W1" s="26"/>
     </row>
@@ -2968,11 +2890,11 @@
         <v>79</v>
       </c>
       <c r="S3" s="34"/>
-      <c r="T3" s="124">
+      <c r="T3" s="123">
         <v>6000000</v>
       </c>
       <c r="U3" s="34" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="V3" s="26"/>
       <c r="W3" s="26"/>
@@ -3034,11 +2956,11 @@
       <c r="T4" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="U4" s="127">
+      <c r="U4" s="126">
         <v>13740903</v>
       </c>
       <c r="V4" s="26" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="W4" s="26"/>
     </row>
@@ -3508,11 +3430,11 @@
       <c r="T12" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="U12" s="127">
+      <c r="U12" s="126">
         <v>4000000</v>
       </c>
       <c r="V12" s="26" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="W12" s="26"/>
     </row>
@@ -3689,11 +3611,11 @@
       <c r="T15" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="U15" s="127">
+      <c r="U15" s="126">
         <v>10000000</v>
       </c>
       <c r="V15" s="26" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="W15" s="26"/>
     </row>
@@ -4005,7 +3927,7 @@
         <v>16</v>
       </c>
       <c r="F21" s="37" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="G21" s="38" t="s">
         <v>79</v>
@@ -4046,7 +3968,7 @@
         <v>120</v>
       </c>
       <c r="U21" s="34" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="V21" s="26"/>
       <c r="W21" s="26"/>
@@ -4068,7 +3990,7 @@
         <v>22</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="G22" s="38" t="s">
         <v>77</v>
@@ -4107,7 +4029,7 @@
         <v>123</v>
       </c>
       <c r="U22" s="34" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="V22" s="26"/>
       <c r="W22" s="26"/>
@@ -4414,7 +4336,7 @@
         <v>31</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="G28" s="38" t="s">
         <v>77</v>
@@ -4451,7 +4373,7 @@
         <v>123</v>
       </c>
       <c r="U28" s="34" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="V28" s="26"/>
       <c r="W28" s="26"/>
@@ -4461,7 +4383,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>239</v>
+        <v>224</v>
       </c>
       <c r="C29" s="35" t="s">
         <v>137</v>
@@ -4473,7 +4395,7 @@
         <v>30</v>
       </c>
       <c r="F29" s="37" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="G29" s="38" t="s">
         <v>77</v>
@@ -4509,11 +4431,11 @@
       <c r="T29" s="46" t="s">
         <v>138</v>
       </c>
-      <c r="U29" s="127">
+      <c r="U29" s="126">
         <v>7365024</v>
       </c>
       <c r="V29" s="26" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="W29" s="26"/>
     </row>
@@ -4852,19 +4774,19 @@
       <c r="W35" s="26"/>
     </row>
     <row r="36" spans="1:23" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="128">
+      <c r="A36" s="127">
         <v>35</v>
       </c>
-      <c r="B36" s="129" t="s">
-        <v>242</v>
-      </c>
-      <c r="C36" s="130" t="s">
+      <c r="B36" s="128" t="s">
+        <v>227</v>
+      </c>
+      <c r="C36" s="129" t="s">
         <v>155</v>
       </c>
-      <c r="D36" s="131">
+      <c r="D36" s="130">
         <v>45950</v>
       </c>
-      <c r="E36" s="132">
+      <c r="E36" s="131">
         <v>39</v>
       </c>
       <c r="F36" s="47" t="s">
@@ -4941,11 +4863,11 @@
       <c r="T37" s="63" t="s">
         <v>159</v>
       </c>
-      <c r="U37" s="133">
+      <c r="U37" s="132">
         <v>40000000</v>
       </c>
       <c r="V37" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="W37" s="26"/>
     </row>
@@ -5035,7 +4957,7 @@
       <c r="C40" s="26"/>
       <c r="D40" s="26"/>
       <c r="E40" s="26"/>
-      <c r="F40" s="125"/>
+      <c r="F40" s="124"/>
       <c r="G40" s="26"/>
       <c r="H40" s="26"/>
       <c r="I40" s="26"/>
@@ -5060,7 +4982,7 @@
       <c r="C41" s="26"/>
       <c r="D41" s="26"/>
       <c r="E41" s="26"/>
-      <c r="F41" s="125"/>
+      <c r="F41" s="124"/>
       <c r="G41" s="26"/>
       <c r="H41" s="26"/>
       <c r="I41" s="26"/>
@@ -5085,7 +5007,7 @@
       <c r="C42" s="26"/>
       <c r="D42" s="26"/>
       <c r="E42" s="26"/>
-      <c r="F42" s="125"/>
+      <c r="F42" s="124"/>
       <c r="G42" s="26"/>
       <c r="H42" s="26"/>
       <c r="I42" s="26"/>
@@ -5114,7 +5036,7 @@
       <c r="C43" s="26"/>
       <c r="D43" s="26"/>
       <c r="E43" s="26"/>
-      <c r="F43" s="125"/>
+      <c r="F43" s="124"/>
       <c r="G43" s="26"/>
       <c r="H43" s="26"/>
       <c r="I43" s="26"/>
@@ -5139,7 +5061,7 @@
       <c r="C44" s="26"/>
       <c r="D44" s="26"/>
       <c r="E44" s="26"/>
-      <c r="F44" s="125"/>
+      <c r="F44" s="124"/>
       <c r="G44" s="26"/>
       <c r="H44" s="26"/>
       <c r="I44" s="26"/>
@@ -5169,38 +5091,39 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E414C69-42B0-4AEA-B31D-03EC12BDB0B7}">
-  <dimension ref="A1:W39"/>
+  <dimension ref="A1:V38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19.26953125" customWidth="1"/>
     <col min="3" max="3" width="17.81640625" customWidth="1"/>
+    <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="21" customWidth="1"/>
     <col min="19" max="19" width="13.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="140"/>
-      <c r="B1" s="141"/>
-      <c r="C1" s="141"/>
-      <c r="D1" s="141"/>
-      <c r="E1" s="141"/>
-      <c r="F1" s="141"/>
-      <c r="G1" s="141"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="141"/>
-      <c r="J1" s="141"/>
-      <c r="K1" s="141"/>
-      <c r="L1" s="141"/>
-      <c r="M1" s="141"/>
-      <c r="N1" s="141"/>
-      <c r="O1" s="141"/>
-      <c r="P1" s="141"/>
-      <c r="Q1" s="141"/>
-      <c r="R1" s="141"/>
-      <c r="S1" s="141"/>
-      <c r="T1" s="141"/>
-      <c r="U1" s="141"/>
-      <c r="V1" s="142"/>
+      <c r="A1" s="139"/>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
+      <c r="P1" s="140"/>
+      <c r="Q1" s="140"/>
+      <c r="R1" s="140"/>
+      <c r="S1" s="140"/>
+      <c r="T1" s="140"/>
+      <c r="U1" s="140"/>
+      <c r="V1" s="141"/>
     </row>
     <row r="2" spans="1:22" ht="25" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="73" t="s">
@@ -5293,7 +5216,9 @@
       <c r="H3" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I3" s="14"/>
+      <c r="I3" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J3" s="14"/>
       <c r="K3" s="59">
         <v>46069</v>
@@ -5335,7 +5260,9 @@
         <v>79</v>
       </c>
       <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
+      <c r="I4" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
       <c r="L4" s="14"/>
@@ -5360,7 +5287,7 @@
         <v>175</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="D5" s="61">
         <v>3</v>
@@ -5373,7 +5300,9 @@
         <v>77</v>
       </c>
       <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
+      <c r="I5" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J5" s="14"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
@@ -5398,7 +5327,7 @@
         <v>132</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="D6" s="61">
         <v>4</v>
@@ -5409,7 +5338,9 @@
       <c r="F6" s="14"/>
       <c r="G6" s="71"/>
       <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
+      <c r="I6" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J6" s="14"/>
       <c r="K6" s="3"/>
       <c r="L6" s="14"/>
@@ -5445,7 +5376,9 @@
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
+      <c r="I7" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
       <c r="L7" s="14"/>
@@ -5485,7 +5418,9 @@
       <c r="H8" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="14"/>
+      <c r="I8" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J8" s="14"/>
       <c r="K8" s="59">
         <v>46069</v>
@@ -5527,7 +5462,9 @@
         <v>79</v>
       </c>
       <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
+      <c r="I9" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J9" s="14"/>
       <c r="K9" s="59">
         <v>46097</v>
@@ -5567,7 +5504,9 @@
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
+      <c r="I10" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -5592,7 +5531,7 @@
         <v>178</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="D11" s="61">
         <v>9</v>
@@ -5603,7 +5542,9 @@
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
+      <c r="I11" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
       <c r="L11" s="14"/>
@@ -5628,7 +5569,7 @@
         <v>179</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="D12" s="61">
         <v>10</v>
@@ -5639,7 +5580,9 @@
       <c r="F12" s="71"/>
       <c r="G12" s="71"/>
       <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
+      <c r="I12" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
       <c r="L12" s="14"/>
@@ -5664,13 +5607,13 @@
         <v>83</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="D13" s="61">
         <v>11</v>
       </c>
       <c r="E13" s="61" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="F13" s="71"/>
       <c r="G13" s="61" t="s">
@@ -5679,7 +5622,9 @@
       <c r="H13" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I13" s="14"/>
+      <c r="I13" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J13" s="14"/>
       <c r="K13" s="14"/>
       <c r="L13" s="14"/>
@@ -5721,9 +5666,11 @@
       <c r="H14" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I14" s="14"/>
+      <c r="I14" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J14" s="14" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="K14" s="59">
         <v>46069</v>
@@ -5767,7 +5714,9 @@
       <c r="H15" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I15" s="14"/>
+      <c r="I15" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J15" s="14"/>
       <c r="K15" s="59">
         <v>46069</v>
@@ -5796,7 +5745,7 @@
         <v>160</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="D16" s="61">
         <v>14</v>
@@ -5811,7 +5760,9 @@
       <c r="H16" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I16" s="14"/>
+      <c r="I16" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
       <c r="L16" s="14"/>
@@ -5849,7 +5800,9 @@
       <c r="H17" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I17" s="14"/>
+      <c r="I17" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J17" s="14"/>
       <c r="K17" s="59">
         <v>46069</v>
@@ -5889,7 +5842,9 @@
       <c r="F18" s="14"/>
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
+      <c r="I18" s="14" t="s">
+        <v>232</v>
+      </c>
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
@@ -5906,7 +5861,7 @@
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
     </row>
-    <row r="19" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="76">
         <v>17</v>
       </c>
@@ -5914,7 +5869,7 @@
         <v>125</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="D19" s="61">
         <v>21</v>
@@ -5927,7 +5882,9 @@
         <v>79</v>
       </c>
       <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
+      <c r="I19" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J19" s="14"/>
       <c r="K19" s="59">
         <v>46097</v>
@@ -5948,7 +5905,7 @@
       <c r="U19" s="3"/>
       <c r="V19" s="3"/>
     </row>
-    <row r="20" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="76">
         <v>18</v>
       </c>
@@ -5969,7 +5926,9 @@
         <v>79</v>
       </c>
       <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="I20" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J20" s="14"/>
       <c r="K20" s="59">
         <v>46097</v>
@@ -6032,7 +5991,7 @@
         <v>184</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="D22" s="61">
         <v>27</v>
@@ -6049,9 +6008,11 @@
       <c r="H22" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I22" s="14"/>
+      <c r="I22" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="J22" s="14" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="K22" s="59">
         <v>46070</v>
@@ -6098,454 +6059,21 @@
       <c r="U23" s="26"/>
       <c r="V23" s="26"/>
     </row>
-    <row r="24" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="26"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="26"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="26"/>
-      <c r="L24" s="26"/>
-      <c r="M24" s="26"/>
-      <c r="N24" s="26"/>
-      <c r="O24" s="26"/>
-      <c r="P24" s="26"/>
-      <c r="Q24" s="26"/>
-      <c r="R24" s="26"/>
-      <c r="S24" s="26"/>
-      <c r="T24" s="26"/>
-      <c r="U24" s="26"/>
-      <c r="V24" s="26"/>
-    </row>
-    <row r="25" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="68"/>
-      <c r="B25" s="68"/>
-      <c r="C25" s="68"/>
-      <c r="D25" s="68"/>
-      <c r="E25" s="68"/>
-      <c r="F25" s="68"/>
-      <c r="G25" s="68"/>
-      <c r="H25" s="68"/>
-      <c r="I25" s="68"/>
-      <c r="J25" s="68"/>
-      <c r="K25" s="68"/>
-      <c r="L25" s="68"/>
-      <c r="M25" s="68"/>
-      <c r="N25" s="68"/>
-      <c r="O25" s="68"/>
-      <c r="P25" s="68"/>
-      <c r="Q25" s="68"/>
-      <c r="R25" s="68"/>
-      <c r="S25" s="68"/>
-      <c r="T25" s="68"/>
-      <c r="U25" s="68"/>
-      <c r="V25" s="68"/>
-    </row>
-    <row r="26" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="143" t="s">
-        <v>185</v>
-      </c>
-      <c r="B26" s="144"/>
-      <c r="C26" s="144"/>
-      <c r="D26" s="144"/>
-      <c r="E26" s="144"/>
-      <c r="F26" s="144"/>
-      <c r="G26" s="144"/>
-      <c r="H26" s="144"/>
-      <c r="I26" s="144"/>
-      <c r="J26" s="144"/>
-      <c r="K26" s="144"/>
-      <c r="L26" s="144"/>
-      <c r="M26" s="144"/>
-      <c r="N26" s="144"/>
-      <c r="O26" s="144"/>
-      <c r="P26" s="144"/>
-      <c r="Q26" s="144"/>
-      <c r="R26" s="144"/>
-      <c r="S26" s="144"/>
-      <c r="T26" s="144"/>
-      <c r="U26" s="144"/>
-      <c r="V26" s="145"/>
-    </row>
-    <row r="27" spans="1:22" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="1"/>
-      <c r="B27" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="3"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="146" t="s">
-        <v>188</v>
-      </c>
-      <c r="S27" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="T27" s="3"/>
-      <c r="U27" s="3"/>
-      <c r="V27" s="3"/>
-    </row>
-    <row r="28" spans="1:22" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="1"/>
-      <c r="B28" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C28" s="149" t="s">
-        <v>190</v>
-      </c>
-      <c r="D28" s="3"/>
-      <c r="E28" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="147"/>
-      <c r="S28" s="3"/>
-      <c r="T28" s="3"/>
-      <c r="U28" s="3"/>
-      <c r="V28" s="3"/>
-    </row>
-    <row r="29" spans="1:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="1"/>
-      <c r="B29" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C29" s="150"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="N29" s="3"/>
-      <c r="O29" s="3"/>
-      <c r="P29" s="3"/>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="147"/>
-      <c r="S29" s="3"/>
-      <c r="T29" s="3"/>
-      <c r="U29" s="3"/>
-      <c r="V29" s="3"/>
-    </row>
-    <row r="30" spans="1:22" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="1"/>
-      <c r="B30" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C30" s="150"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
-      <c r="M30" s="3"/>
-      <c r="N30" s="3"/>
-      <c r="O30" s="3"/>
-      <c r="P30" s="3"/>
-      <c r="Q30" s="3"/>
-      <c r="R30" s="147"/>
-      <c r="S30" s="3"/>
-      <c r="T30" s="3"/>
-      <c r="U30" s="3"/>
-      <c r="V30" s="3"/>
-    </row>
-    <row r="31" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="1"/>
-      <c r="B31" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="C31" s="150"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
-      <c r="N31" s="3"/>
-      <c r="O31" s="3"/>
-      <c r="P31" s="3"/>
-      <c r="Q31" s="3"/>
-      <c r="R31" s="148"/>
-      <c r="S31" s="3"/>
-      <c r="T31" s="3"/>
-      <c r="U31" s="3"/>
-      <c r="V31" s="3"/>
-    </row>
-    <row r="32" spans="1:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="1"/>
-      <c r="B32" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="C32" s="151"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
-      <c r="N32" s="3"/>
-      <c r="O32" s="3"/>
-      <c r="P32" s="3"/>
-      <c r="Q32" s="3"/>
-      <c r="R32" s="82" t="s">
-        <v>195</v>
-      </c>
-      <c r="S32" s="3"/>
-      <c r="T32" s="3"/>
-      <c r="U32" s="3"/>
-      <c r="V32" s="3"/>
-    </row>
-    <row r="33" spans="1:23" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="1"/>
-      <c r="B33" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="D33" s="3"/>
-      <c r="E33" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="3"/>
-      <c r="O33" s="3"/>
-      <c r="P33" s="3"/>
-      <c r="Q33" s="3"/>
-      <c r="R33" s="3"/>
-      <c r="S33" s="3"/>
-      <c r="T33" s="3"/>
-      <c r="U33" s="3"/>
-      <c r="V33" s="3"/>
-    </row>
-    <row r="34" spans="1:23" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="1"/>
-      <c r="B34" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
-      <c r="O34" s="3"/>
-      <c r="P34" s="3"/>
-      <c r="Q34" s="3"/>
-      <c r="R34" s="3"/>
-      <c r="S34" s="3"/>
-      <c r="T34" s="3"/>
-      <c r="U34" s="3"/>
-      <c r="V34" s="3"/>
-    </row>
-    <row r="35" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="26"/>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="26"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="26"/>
-      <c r="N35" s="26"/>
-      <c r="O35" s="26"/>
-      <c r="P35" s="26"/>
-      <c r="Q35" s="26"/>
-      <c r="R35" s="26"/>
-      <c r="S35" s="26"/>
-      <c r="T35" s="26"/>
-      <c r="U35" s="26"/>
-      <c r="V35" s="26"/>
-    </row>
-    <row r="36" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="68"/>
-      <c r="B36" s="68"/>
-      <c r="C36" s="68"/>
-      <c r="D36" s="68"/>
-      <c r="E36" s="68"/>
-      <c r="F36" s="68"/>
-      <c r="G36" s="68"/>
-      <c r="H36" s="68"/>
-      <c r="I36" s="68"/>
-      <c r="J36" s="68"/>
-      <c r="K36" s="68"/>
-      <c r="L36" s="68"/>
-      <c r="M36" s="68"/>
-      <c r="N36" s="68"/>
-      <c r="O36" s="68"/>
-      <c r="P36" s="68"/>
-      <c r="Q36" s="68"/>
-      <c r="R36" s="68"/>
-      <c r="S36" s="68"/>
-      <c r="T36" s="68"/>
-      <c r="U36" s="68"/>
-      <c r="V36" s="68"/>
-    </row>
-    <row r="37" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="143" t="s">
-        <v>199</v>
-      </c>
-      <c r="B37" s="144"/>
-      <c r="C37" s="144"/>
-      <c r="D37" s="144"/>
-      <c r="E37" s="144"/>
-      <c r="F37" s="144"/>
-      <c r="G37" s="144"/>
-      <c r="H37" s="144"/>
-      <c r="I37" s="144"/>
-      <c r="J37" s="144"/>
-      <c r="K37" s="144"/>
-      <c r="L37" s="144"/>
-      <c r="M37" s="144"/>
-      <c r="N37" s="144"/>
-      <c r="O37" s="144"/>
-      <c r="P37" s="144"/>
-      <c r="Q37" s="144"/>
-      <c r="R37" s="144"/>
-      <c r="S37" s="144"/>
-      <c r="T37" s="144"/>
-      <c r="U37" s="144"/>
-      <c r="V37" s="145"/>
-      <c r="W37" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="38" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="26"/>
-      <c r="B38" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="C38" s="26"/>
-      <c r="D38" s="18" t="s">
-        <v>244</v>
-      </c>
-      <c r="E38" s="26">
-        <v>2024</v>
-      </c>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="26"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
-      <c r="N38" s="26"/>
-      <c r="O38" s="26"/>
-      <c r="P38" s="26"/>
-      <c r="Q38" s="26"/>
-      <c r="R38" s="26"/>
-      <c r="S38" s="26"/>
-      <c r="T38" s="26"/>
-      <c r="U38" s="26"/>
-      <c r="V38" s="26"/>
-    </row>
-    <row r="39" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="26"/>
-      <c r="B39" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="C39" s="26"/>
-      <c r="D39" s="18" t="s">
-        <v>244</v>
-      </c>
-      <c r="E39" s="26">
-        <v>2025</v>
-      </c>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="26"/>
-      <c r="K39" s="26"/>
-      <c r="L39" s="26"/>
-      <c r="M39" s="26"/>
-      <c r="N39" s="26"/>
-      <c r="O39" s="26"/>
-      <c r="P39" s="26"/>
-      <c r="Q39" s="26"/>
-      <c r="R39" s="26"/>
-      <c r="S39" s="26"/>
-      <c r="T39" s="26"/>
-      <c r="U39" s="26"/>
-      <c r="V39" s="26"/>
-    </row>
+    <row r="28" spans="1:22" ht="21.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="33" spans="1:1" ht="32.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="1">
     <mergeCell ref="A1:V1"/>
-    <mergeCell ref="A26:V26"/>
-    <mergeCell ref="R27:R31"/>
-    <mergeCell ref="C28:C32"/>
-    <mergeCell ref="A37:V37"/>
   </mergeCells>
   <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6564,61 +6092,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="82" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="84" t="s">
+      <c r="B1" s="83" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="84" t="s">
-        <v>206</v>
-      </c>
-      <c r="D1" s="84" t="s">
+      <c r="C1" s="83" t="s">
+        <v>191</v>
+      </c>
+      <c r="D1" s="83" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="84" t="s">
-        <v>207</v>
-      </c>
-      <c r="F1" s="84" t="s">
+      <c r="E1" s="83" t="s">
+        <v>192</v>
+      </c>
+      <c r="F1" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="84" t="s">
+      <c r="G1" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="84" t="s">
+      <c r="H1" s="83" t="s">
         <v>168</v>
       </c>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="J1" s="84" t="s">
+      <c r="J1" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="K1" s="84" t="s">
+      <c r="K1" s="83" t="s">
         <v>66</v>
       </c>
-      <c r="L1" s="84" t="s">
+      <c r="L1" s="83" t="s">
         <v>67</v>
       </c>
-      <c r="M1" s="84" t="s">
+      <c r="M1" s="83" t="s">
         <v>68</v>
       </c>
-      <c r="N1" s="84" t="s">
+      <c r="N1" s="83" t="s">
         <v>70</v>
       </c>
-      <c r="O1" s="84" t="s">
+      <c r="O1" s="83" t="s">
         <v>71</v>
       </c>
-      <c r="P1" s="84" t="s">
+      <c r="P1" s="83" t="s">
         <v>169</v>
       </c>
-      <c r="Q1" s="84" t="s">
+      <c r="Q1" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="R1" s="85" t="s">
+      <c r="R1" s="84" t="s">
         <v>170</v>
       </c>
-      <c r="S1" s="85" t="s">
+      <c r="S1" s="84" t="s">
         <v>171</v>
       </c>
     </row>
@@ -6626,23 +6154,23 @@
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="86" t="s">
-        <v>208</v>
+      <c r="B2" s="85" t="s">
+        <v>193</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="87">
+      <c r="I2" s="86">
         <v>46070</v>
       </c>
-      <c r="J2" s="88">
+      <c r="J2" s="87">
         <v>46250</v>
       </c>
       <c r="K2" s="3"/>
@@ -6650,7 +6178,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
-      <c r="P2" s="89">
+      <c r="P2" s="88">
         <v>30000000</v>
       </c>
       <c r="Q2" s="3"/>
@@ -6661,23 +6189,23 @@
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="86" t="s">
-        <v>211</v>
+      <c r="B3" s="85" t="s">
+        <v>196</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="87">
+      <c r="I3" s="86">
         <v>46071</v>
       </c>
-      <c r="J3" s="88">
+      <c r="J3" s="87">
         <v>46251</v>
       </c>
       <c r="K3" s="3"/>
@@ -6685,7 +6213,7 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
-      <c r="P3" s="89">
+      <c r="P3" s="88">
         <v>30000000</v>
       </c>
       <c r="Q3" s="3"/>
@@ -6696,14 +6224,14 @@
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="86" t="s">
-        <v>214</v>
+      <c r="B4" s="85" t="s">
+        <v>199</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -6716,7 +6244,7 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
-      <c r="P4" s="89">
+      <c r="P4" s="88">
         <v>30000000</v>
       </c>
       <c r="Q4" s="3"/>
@@ -6727,14 +6255,14 @@
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="86" t="s">
-        <v>217</v>
+      <c r="B5" s="85" t="s">
+        <v>202</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -6747,7 +6275,7 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
-      <c r="P5" s="89">
+      <c r="P5" s="88">
         <v>30000000</v>
       </c>
       <c r="Q5" s="3"/>
@@ -6755,30 +6283,30 @@
       <c r="S5" s="3"/>
     </row>
     <row r="6" spans="1:19" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="97">
+      <c r="A6" s="96">
         <v>5</v>
       </c>
-      <c r="B6" s="98" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="99" t="s">
-        <v>221</v>
-      </c>
-      <c r="D6" s="99" t="s">
-        <v>222</v>
-      </c>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="100"/>
-      <c r="L6" s="100"/>
-      <c r="M6" s="100"/>
-      <c r="N6" s="100"/>
-      <c r="O6" s="100"/>
-      <c r="P6" s="89">
+      <c r="B6" s="97" t="s">
+        <v>205</v>
+      </c>
+      <c r="C6" s="98" t="s">
+        <v>206</v>
+      </c>
+      <c r="D6" s="98" t="s">
+        <v>207</v>
+      </c>
+      <c r="E6" s="99"/>
+      <c r="F6" s="99"/>
+      <c r="G6" s="99"/>
+      <c r="H6" s="99"/>
+      <c r="I6" s="99"/>
+      <c r="J6" s="99"/>
+      <c r="K6" s="99"/>
+      <c r="L6" s="99"/>
+      <c r="M6" s="99"/>
+      <c r="N6" s="99"/>
+      <c r="O6" s="99"/>
+      <c r="P6" s="88">
         <v>30000000</v>
       </c>
       <c r="Q6" s="3"/>
@@ -6786,136 +6314,136 @@
       <c r="S6" s="3"/>
     </row>
     <row r="7" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="101">
+      <c r="A7" s="100">
         <v>6</v>
       </c>
-      <c r="B7" s="102" t="s">
-        <v>223</v>
-      </c>
-      <c r="C7" s="103" t="s">
-        <v>224</v>
-      </c>
-      <c r="D7" s="103" t="s">
-        <v>225</v>
-      </c>
-      <c r="E7" s="104"/>
-      <c r="F7" s="104"/>
-      <c r="G7" s="104"/>
-      <c r="H7" s="104"/>
-      <c r="I7" s="105">
+      <c r="B7" s="101" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7" s="102" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="102" t="s">
+        <v>210</v>
+      </c>
+      <c r="E7" s="103"/>
+      <c r="F7" s="103"/>
+      <c r="G7" s="103"/>
+      <c r="H7" s="103"/>
+      <c r="I7" s="104">
         <v>46071</v>
       </c>
-      <c r="J7" s="106">
+      <c r="J7" s="105">
         <v>46251</v>
       </c>
-      <c r="K7" s="104"/>
-      <c r="L7" s="104"/>
-      <c r="M7" s="104"/>
-      <c r="N7" s="104"/>
-      <c r="O7" s="104"/>
-      <c r="P7" s="116">
+      <c r="K7" s="103"/>
+      <c r="L7" s="103"/>
+      <c r="M7" s="103"/>
+      <c r="N7" s="103"/>
+      <c r="O7" s="103"/>
+      <c r="P7" s="115">
         <v>30000000</v>
       </c>
-      <c r="Q7" s="110"/>
-      <c r="R7" s="111"/>
-      <c r="S7" s="111"/>
+      <c r="Q7" s="109"/>
+      <c r="R7" s="110"/>
+      <c r="S7" s="110"/>
     </row>
     <row r="8" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="92"/>
-      <c r="B8" s="93"/>
-      <c r="C8" s="92"/>
-      <c r="D8" s="92"/>
-      <c r="E8" s="94"/>
-      <c r="F8" s="94"/>
-      <c r="G8" s="94"/>
-      <c r="H8" s="94"/>
-      <c r="I8" s="95"/>
-      <c r="J8" s="96"/>
-      <c r="K8" s="94"/>
-      <c r="L8" s="94"/>
-      <c r="M8" s="94"/>
-      <c r="N8" s="94"/>
-      <c r="O8" s="94"/>
-      <c r="P8" s="109"/>
-      <c r="Q8" s="94"/>
-      <c r="R8" s="94"/>
-      <c r="S8" s="94"/>
+      <c r="A8" s="91"/>
+      <c r="B8" s="92"/>
+      <c r="C8" s="91"/>
+      <c r="D8" s="91"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="94"/>
+      <c r="J8" s="95"/>
+      <c r="K8" s="93"/>
+      <c r="L8" s="93"/>
+      <c r="M8" s="93"/>
+      <c r="N8" s="93"/>
+      <c r="O8" s="93"/>
+      <c r="P8" s="108"/>
+      <c r="Q8" s="93"/>
+      <c r="R8" s="93"/>
+      <c r="S8" s="93"/>
     </row>
     <row r="9" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="92"/>
-      <c r="B9" s="93"/>
-      <c r="C9" s="92"/>
-      <c r="D9" s="92"/>
-      <c r="E9" s="94"/>
-      <c r="F9" s="94"/>
-      <c r="G9" s="94"/>
-      <c r="H9" s="94"/>
-      <c r="I9" s="95"/>
-      <c r="J9" s="96"/>
-      <c r="K9" s="94"/>
-      <c r="L9" s="94"/>
-      <c r="M9" s="94"/>
-      <c r="N9" s="94"/>
-      <c r="O9" s="94"/>
-      <c r="P9" s="109"/>
-      <c r="Q9" s="94"/>
-      <c r="R9" s="94"/>
-      <c r="S9" s="94"/>
+      <c r="A9" s="91"/>
+      <c r="B9" s="92"/>
+      <c r="C9" s="91"/>
+      <c r="D9" s="91"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="94"/>
+      <c r="J9" s="95"/>
+      <c r="K9" s="93"/>
+      <c r="L9" s="93"/>
+      <c r="M9" s="93"/>
+      <c r="N9" s="93"/>
+      <c r="O9" s="93"/>
+      <c r="P9" s="108"/>
+      <c r="Q9" s="93"/>
+      <c r="R9" s="93"/>
+      <c r="S9" s="93"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A10" s="94"/>
-      <c r="B10" s="94"/>
-      <c r="C10" s="94"/>
-      <c r="D10" s="94"/>
-      <c r="E10" s="94"/>
-      <c r="F10" s="94"/>
-      <c r="G10" s="94"/>
-      <c r="H10" s="94"/>
-      <c r="I10" s="94"/>
-      <c r="J10" s="94"/>
-      <c r="K10" s="94"/>
-      <c r="L10" s="94"/>
-      <c r="M10" s="94"/>
-      <c r="N10" s="94"/>
-      <c r="O10" s="94"/>
-      <c r="Q10" s="94"/>
-      <c r="R10" s="94"/>
-      <c r="S10" s="94"/>
+      <c r="A10" s="93"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
+      <c r="H10" s="93"/>
+      <c r="I10" s="93"/>
+      <c r="J10" s="93"/>
+      <c r="K10" s="93"/>
+      <c r="L10" s="93"/>
+      <c r="M10" s="93"/>
+      <c r="N10" s="93"/>
+      <c r="O10" s="93"/>
+      <c r="Q10" s="93"/>
+      <c r="R10" s="93"/>
+      <c r="S10" s="93"/>
     </row>
     <row r="11" spans="1:19" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="91"/>
-      <c r="B11" s="112" t="s">
-        <v>226</v>
-      </c>
-      <c r="C11" s="113" t="s">
-        <v>227</v>
-      </c>
-      <c r="D11" s="114"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="114"/>
-      <c r="G11" s="114"/>
-      <c r="H11" s="114"/>
-      <c r="I11" s="114"/>
-      <c r="J11" s="114"/>
-      <c r="K11" s="114"/>
-      <c r="L11" s="114"/>
-      <c r="M11" s="114"/>
-      <c r="N11" s="114"/>
-      <c r="O11" s="114"/>
-      <c r="P11" s="115">
+      <c r="A11" s="90"/>
+      <c r="B11" s="111" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" s="112" t="s">
+        <v>212</v>
+      </c>
+      <c r="D11" s="113"/>
+      <c r="E11" s="113"/>
+      <c r="F11" s="113"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="113"/>
+      <c r="L11" s="113"/>
+      <c r="M11" s="113"/>
+      <c r="N11" s="113"/>
+      <c r="O11" s="113"/>
+      <c r="P11" s="114">
         <v>30000000</v>
       </c>
-      <c r="Q11" s="114"/>
-      <c r="R11" s="114"/>
-      <c r="S11" s="114"/>
+      <c r="Q11" s="113"/>
+      <c r="R11" s="113"/>
+      <c r="S11" s="113"/>
     </row>
     <row r="12" spans="1:19" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1"/>
       <c r="B12" s="4" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -6929,7 +6457,7 @@
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
-      <c r="P12" s="89">
+      <c r="P12" s="88">
         <v>30000000</v>
       </c>
       <c r="Q12" s="3"/>
@@ -6952,7 +6480,7 @@
       <c r="M13" s="68"/>
       <c r="N13" s="68"/>
       <c r="O13" s="68"/>
-      <c r="P13" s="89"/>
+      <c r="P13" s="88"/>
       <c r="Q13" s="68"/>
       <c r="R13" s="68"/>
       <c r="S13" s="26"/>
@@ -6963,7 +6491,7 @@
         <v>185</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -6977,7 +6505,7 @@
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
-      <c r="P14" s="89">
+      <c r="P14" s="88">
         <v>30000000</v>
       </c>
       <c r="Q14" s="3"/>
@@ -6986,11 +6514,11 @@
     </row>
     <row r="15" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1"/>
-      <c r="B15" s="152" t="s">
+      <c r="B15" s="142" t="s">
         <v>185</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
@@ -7004,7 +6532,7 @@
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
-      <c r="P15" s="89">
+      <c r="P15" s="88">
         <v>30000000</v>
       </c>
       <c r="Q15" s="3"/>
@@ -7013,9 +6541,9 @@
     </row>
     <row r="16" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1"/>
-      <c r="B16" s="153"/>
+      <c r="B16" s="143"/>
       <c r="C16" s="4" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
@@ -7029,7 +6557,7 @@
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
-      <c r="P16" s="89">
+      <c r="P16" s="88">
         <v>30000000</v>
       </c>
       <c r="Q16" s="3"/>
@@ -7038,9 +6566,9 @@
     </row>
     <row r="17" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1"/>
-      <c r="B17" s="153"/>
+      <c r="B17" s="143"/>
       <c r="C17" s="4" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -7054,7 +6582,7 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
-      <c r="P17" s="89">
+      <c r="P17" s="88">
         <v>30000000</v>
       </c>
       <c r="Q17" s="3"/>
@@ -7063,9 +6591,9 @@
     </row>
     <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1"/>
-      <c r="B18" s="154"/>
+      <c r="B18" s="144"/>
       <c r="C18" s="4" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -7079,7 +6607,7 @@
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
-      <c r="P18" s="107">
+      <c r="P18" s="106">
         <v>30000000</v>
       </c>
       <c r="Q18" s="3"/>
@@ -7101,12 +6629,12 @@
       <c r="L19" s="26"/>
       <c r="M19" s="26"/>
       <c r="N19" s="26"/>
-      <c r="O19" s="117"/>
-      <c r="P19" s="108">
+      <c r="O19" s="116"/>
+      <c r="P19" s="107">
         <f>SUM(P2:P18)</f>
         <v>390000000</v>
       </c>
-      <c r="Q19" s="118"/>
+      <c r="Q19" s="117"/>
       <c r="R19" s="26"/>
       <c r="S19" s="26"/>
     </row>
@@ -7126,7 +6654,7 @@
       <c r="M20" s="26"/>
       <c r="N20" s="26"/>
       <c r="O20" s="26"/>
-      <c r="P20" s="119"/>
+      <c r="P20" s="118"/>
       <c r="Q20" s="26"/>
       <c r="R20" s="26"/>
       <c r="S20" s="26"/>
@@ -7199,10 +6727,10 @@
     <row r="24" spans="1:19" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="26"/>
       <c r="B24" s="18" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="D24" s="26"/>
       <c r="E24" s="26"/>
@@ -7243,9 +6771,9 @@
       <c r="S25" s="26"/>
     </row>
     <row r="26" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="90"/>
+      <c r="A26" s="89"/>
       <c r="B26" s="4" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="C26" s="26"/>
       <c r="D26" s="26"/>
@@ -7266,9 +6794,9 @@
       <c r="S26" s="26"/>
     </row>
     <row r="27" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="90"/>
+      <c r="A27" s="89"/>
       <c r="B27" s="4" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="C27" s="26"/>
       <c r="D27" s="26"/>

</xml_diff>